<commit_message>
Add multimodal retrieval evaluation pipeline
</commit_message>
<xml_diff>
--- a/data/evaluation/testset.xlsx
+++ b/data/evaluation/testset.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d271c3618886ac09/Desktop/my_research/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\OneDrive\Desktop\Multimodal-Offline-RAG-System\data\evaluation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="11_4AFF9AC6A2A3E4D7B0FDAF44048FE453F0D02119" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5BCD272E-CEC3-48A4-BFE4-9F8D3D7B216A}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CECA6C88-9477-47B3-B6BE-762F0A0C63CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="11520" windowHeight="12360" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2280" yWindow="2280" windowWidth="19200" windowHeight="11170" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -470,12 +470,6 @@
     <t>page_155_img_1_0.jpeg</t>
   </si>
   <si>
-    <t>Qwen2.5:1.5b</t>
-  </si>
-  <si>
-    <t>Gemma 2.5:2B</t>
-  </si>
-  <si>
     <t>text</t>
   </si>
   <si>
@@ -483,6 +477,14 @@
   </si>
   <si>
     <t>로봇 케이블을 임의로 개조하거나 연장할 경우 발생할 수 있는 가장 큰 위험 두 가지는 무엇입니까?</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Qwen2.5</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Gemma 2.5</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -816,14 +818,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A2:E40"/>
-  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="116.09765625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="48.3984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="116.08203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="48.4140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
       <c r="B2" t="s">
         <v>0</v>
       </c>
@@ -837,12 +839,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>5</v>
@@ -854,7 +856,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
@@ -871,7 +873,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
@@ -888,7 +890,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>14</v>
       </c>
@@ -905,7 +907,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>18</v>
       </c>
@@ -922,7 +924,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>22</v>
       </c>
@@ -939,7 +941,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
         <v>26</v>
       </c>
@@ -956,7 +958,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A10" s="1" t="s">
         <v>30</v>
       </c>
@@ -973,7 +975,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="11" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A11" s="1" t="s">
         <v>34</v>
       </c>
@@ -990,7 +992,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A12" s="1" t="s">
         <v>37</v>
       </c>
@@ -1007,7 +1009,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="13" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A13" s="1" t="s">
         <v>41</v>
       </c>
@@ -1024,7 +1026,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="14" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A14" s="1" t="s">
         <v>45</v>
       </c>
@@ -1041,7 +1043,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="15" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A15" s="1" t="s">
         <v>49</v>
       </c>
@@ -1058,7 +1060,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="16" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A16" s="1" t="s">
         <v>53</v>
       </c>
@@ -1075,7 +1077,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="17" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A17" s="1" t="s">
         <v>57</v>
       </c>
@@ -1092,7 +1094,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="18" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A18" s="1" t="s">
         <v>61</v>
       </c>
@@ -1109,7 +1111,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="19" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A19" s="1" t="s">
         <v>65</v>
       </c>
@@ -1126,7 +1128,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="20" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A20" s="1" t="s">
         <v>68</v>
       </c>
@@ -1143,7 +1145,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="21" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A21" s="1" t="s">
         <v>72</v>
       </c>
@@ -1160,7 +1162,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="22" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A22" s="1" t="s">
         <v>76</v>
       </c>
@@ -1177,7 +1179,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="23" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A23" s="1" t="s">
         <v>80</v>
       </c>
@@ -1194,7 +1196,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="24" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A24" s="1" t="s">
         <v>84</v>
       </c>
@@ -1211,7 +1213,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="25" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A25" s="1" t="s">
         <v>88</v>
       </c>
@@ -1228,7 +1230,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="26" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A26" s="1" t="s">
         <v>92</v>
       </c>
@@ -1245,7 +1247,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="27" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A27" s="1" t="s">
         <v>96</v>
       </c>
@@ -1262,7 +1264,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="28" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A28" s="1" t="s">
         <v>99</v>
       </c>
@@ -1279,7 +1281,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="29" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A29" s="1" t="s">
         <v>103</v>
       </c>
@@ -1296,7 +1298,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="30" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A30" s="1" t="s">
         <v>107</v>
       </c>
@@ -1313,7 +1315,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="31" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A31" s="1" t="s">
         <v>111</v>
       </c>
@@ -1330,7 +1332,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="32" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A32" s="1" t="s">
         <v>115</v>
       </c>
@@ -1347,7 +1349,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="33" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A33" s="1" t="s">
         <v>118</v>
       </c>
@@ -1364,7 +1366,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="34" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A34" s="1" t="s">
         <v>121</v>
       </c>
@@ -1381,7 +1383,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="35" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A35" s="1" t="s">
         <v>125</v>
       </c>
@@ -1398,7 +1400,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="36" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A36" s="1" t="s">
         <v>129</v>
       </c>
@@ -1415,7 +1417,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="37" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A37" s="1" t="s">
         <v>133</v>
       </c>
@@ -1432,7 +1434,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="38" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A38" s="1" t="s">
         <v>137</v>
       </c>
@@ -1449,7 +1451,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="39" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A39" s="1" t="s">
         <v>141</v>
       </c>
@@ -1466,7 +1468,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="40" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A40" s="1" t="s">
         <v>145</v>
       </c>
@@ -1492,37 +1494,37 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E42"/>
-  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="C1" s="3"/>
       <c r="D1" s="2" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="E1" s="3"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A2" s="3"/>
       <c r="B2" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.4">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -1531,7 +1533,7 @@
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
@@ -1540,7 +1542,7 @@
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
@@ -1549,7 +1551,7 @@
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>14</v>
       </c>
@@ -1558,7 +1560,7 @@
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>18</v>
       </c>
@@ -1567,7 +1569,7 @@
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>22</v>
       </c>
@@ -1576,7 +1578,7 @@
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
         <v>26</v>
       </c>
@@ -1585,7 +1587,7 @@
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A10" s="1" t="s">
         <v>30</v>
       </c>
@@ -1594,7 +1596,7 @@
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A11" s="1" t="s">
         <v>34</v>
       </c>
@@ -1603,7 +1605,7 @@
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A12" s="1" t="s">
         <v>37</v>
       </c>
@@ -1612,7 +1614,7 @@
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A13" s="1" t="s">
         <v>41</v>
       </c>
@@ -1621,7 +1623,7 @@
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A14" s="1" t="s">
         <v>45</v>
       </c>
@@ -1630,7 +1632,7 @@
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A15" s="1" t="s">
         <v>49</v>
       </c>
@@ -1639,7 +1641,7 @@
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A16" s="1" t="s">
         <v>53</v>
       </c>
@@ -1648,7 +1650,7 @@
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A17" s="1" t="s">
         <v>57</v>
       </c>
@@ -1657,7 +1659,7 @@
       <c r="D17" s="1"/>
       <c r="E17" s="1"/>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A18" s="1" t="s">
         <v>61</v>
       </c>
@@ -1666,7 +1668,7 @@
       <c r="D18" s="1"/>
       <c r="E18" s="1"/>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A19" s="1" t="s">
         <v>65</v>
       </c>
@@ -1675,7 +1677,7 @@
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A20" s="1" t="s">
         <v>68</v>
       </c>
@@ -1684,7 +1686,7 @@
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A21" s="1" t="s">
         <v>72</v>
       </c>
@@ -1693,7 +1695,7 @@
       <c r="D21" s="1"/>
       <c r="E21" s="1"/>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A22" s="1" t="s">
         <v>76</v>
       </c>
@@ -1702,7 +1704,7 @@
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A23" s="1" t="s">
         <v>80</v>
       </c>
@@ -1711,7 +1713,7 @@
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A24" s="1" t="s">
         <v>84</v>
       </c>
@@ -1720,7 +1722,7 @@
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A25" s="1" t="s">
         <v>88</v>
       </c>
@@ -1729,7 +1731,7 @@
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A26" s="1" t="s">
         <v>92</v>
       </c>
@@ -1738,7 +1740,7 @@
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A27" s="1" t="s">
         <v>96</v>
       </c>
@@ -1747,7 +1749,7 @@
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A28" s="1" t="s">
         <v>99</v>
       </c>
@@ -1756,7 +1758,7 @@
       <c r="D28" s="1"/>
       <c r="E28" s="1"/>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A29" s="1" t="s">
         <v>103</v>
       </c>
@@ -1765,7 +1767,7 @@
       <c r="D29" s="1"/>
       <c r="E29" s="1"/>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A30" s="1" t="s">
         <v>107</v>
       </c>
@@ -1774,7 +1776,7 @@
       <c r="D30" s="1"/>
       <c r="E30" s="1"/>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A31" s="1" t="s">
         <v>111</v>
       </c>
@@ -1783,7 +1785,7 @@
       <c r="D31" s="1"/>
       <c r="E31" s="1"/>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A32" s="1" t="s">
         <v>115</v>
       </c>
@@ -1792,7 +1794,7 @@
       <c r="D32" s="1"/>
       <c r="E32" s="1"/>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A33" s="1" t="s">
         <v>118</v>
       </c>
@@ -1801,7 +1803,7 @@
       <c r="D33" s="1"/>
       <c r="E33" s="1"/>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A34" s="1" t="s">
         <v>121</v>
       </c>
@@ -1810,7 +1812,7 @@
       <c r="D34" s="1"/>
       <c r="E34" s="1"/>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A35" s="1" t="s">
         <v>125</v>
       </c>
@@ -1819,7 +1821,7 @@
       <c r="D35" s="1"/>
       <c r="E35" s="1"/>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A36" s="1" t="s">
         <v>129</v>
       </c>
@@ -1828,7 +1830,7 @@
       <c r="D36" s="1"/>
       <c r="E36" s="1"/>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A37" s="1" t="s">
         <v>133</v>
       </c>
@@ -1837,7 +1839,7 @@
       <c r="D37" s="1"/>
       <c r="E37" s="1"/>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A38" s="1" t="s">
         <v>137</v>
       </c>
@@ -1846,7 +1848,7 @@
       <c r="D38" s="1"/>
       <c r="E38" s="1"/>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A39" s="1" t="s">
         <v>141</v>
       </c>
@@ -1855,7 +1857,7 @@
       <c r="D39" s="1"/>
       <c r="E39" s="1"/>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A40" s="1" t="s">
         <v>145</v>
       </c>
@@ -1864,14 +1866,14 @@
       <c r="D40" s="1"/>
       <c r="E40" s="1"/>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
       <c r="C41" s="1"/>
       <c r="D41" s="1"/>
       <c r="E41" s="1"/>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A42" s="1"/>
       <c r="B42" s="1"/>
       <c r="C42" s="1"/>

</xml_diff>